<commit_message>
Backlog validado contra el despliegue provisional en VPS
</commit_message>
<xml_diff>
--- a/desarollo/PRODUCT BACKLOG_v2_validado.xlsx
+++ b/desarollo/PRODUCT BACKLOG_v2_validado.xlsx
@@ -1000,7 +1000,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Transcribir en el propio servidor, sin enviar el audio a terceros</t>
+          <t>Transcribir sin enviar el audio a terceros</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
@@ -1009,17 +1009,21 @@
       <c r="E14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Validada</t>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Con cambios</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Whisper corre en el servidor</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
+          <t>Salud del sistema: transcripción remota alcanzable</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Whisper corre en la PC del equipo y el VPS le envía el audio por un túnel SSH cifrado; ningún tercero recibe el audio.</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
@@ -3310,12 +3314,12 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Dominio público del VPS</t>
+          <t>http://162.243.33.172:8080</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Entorno provisional para validar con la misma pila de la arquitectura objetivo en Azure; plan y scripts listos, falta ejecutarlos.</t>
+          <t>Publicado en el VPS provisional con la misma pila de la arquitectura objetivo en Azure; falta el subdominio con HTTPS.</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -3537,10 +3541,10 @@
         <v>18</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
         <v>1</v>
@@ -3929,10 +3933,10 @@
         <v>328</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F21" s="9" t="n">
         <v>4</v>

</xml_diff>

<commit_message>
Rediseño de experiencia: landing adaptable, cursos y clases directos y textos para el estudiante
- Landing nueva con tamaños adaptables y vista previa del plan de hoy
- Nuevo curso en una pantalla corta con detalles opcionales plegados
- Página del curso con acciones arriba, clases primero y columna lateral
- Nueva clase con selector texto/audio, zona para soltar el audio y grabador con colores de marca
- Mis cursos abre con saludo compacto y tarjetas de cursos
- Textos sin jerga técnica en pantallas y mensajes
- Estilos en static/learning/css/redesign.css con soporte de modo oscuro
- Pruebas actualizadas al nuevo texto; backlog validado con la épica Experiencia de uso
</commit_message>
<xml_diff>
--- a/desarollo/PRODUCT BACKLOG_v2_validado.xlsx
+++ b/desarollo/PRODUCT BACKLOG_v2_validado.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backlog validado'!$A$1:$I$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backlog validado'!$A$1:$I$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -658,7 +658,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Dashboard → Preferencias</t>
+          <t>Mis cursos → Preferencias</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Panel lateral y dashboard</t>
+          <t>Panel lateral y Mis cursos</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -732,7 +732,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Nuevo curso</t>
+          <t>Mis cursos → Nuevo curso</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -767,7 +767,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Editar curso → Archivar</t>
+          <t>Curso → menú ··· → Archivar</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -911,7 +911,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Dashboard → Explorar</t>
+          <t>Mis cursos → Explorar</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -946,10 +946,14 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Página de inicio</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
+          <t>Página de inicio en computadora y celular</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Rediseñada en septiembre de 2026: mensaje corto, vista previa del plan de hoy y diseño adaptable.</t>
+        </is>
+      </c>
       <c r="I12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1090,7 +1094,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Ver pipeline: etapa, hora y detalle</t>
+          <t>Clase → Ver estado: etapa, hora y detalle</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -1164,12 +1168,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Nueva clase: selector de dónde generar</t>
+          <t>Nueva clase → Opciones → Generar con</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>En el servidor solo hay nube (Groq); la opción local se desactiva cuando no hay modelo local.</t>
+          <t>La opción solo aparece si hay dos motores; en el servidor solo hay nube (Groq).</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1203,7 +1207,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Nueva clase: selector de verificación</t>
+          <t>Nueva clase → Opciones → Revisar preguntas con</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -1273,7 +1277,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Nueva clase: costo estimado</t>
+          <t>Nueva clase: «Usa unos N créditos» junto al botón</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -2320,7 +2324,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Dashboard: racha</t>
+          <t>Mis cursos: racha junto al saludo</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -2355,7 +2359,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Curso: recomendaciones con hecha o descartar</t>
+          <t>Curso: recomendaciones con Hecho u Omitir</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -2638,7 +2642,11 @@
           <t>Clase → Descargar</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Se descarga como «Copia de tus preguntas».</t>
+        </is>
+      </c>
       <c r="I59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
@@ -2869,7 +2877,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Práctica terminada → Generar refuerzo</t>
+          <t>Práctica terminada → Generar refuerzo · Curso → Crear material de refuerzo</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -2951,7 +2959,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Dashboard: Hoy en SIMA</t>
+          <t>Mis cursos: Hoy en SIMA · Curso: Plan de hoy</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -2990,7 +2998,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Curso → Temas en riesgo</t>
+          <t>Curso → Estudiar → Repasar antes de olvidar</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -3029,7 +3037,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Curso → Simulacro</t>
+          <t>Curso → Estudiar → Simulacro</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -3068,7 +3076,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Dashboard: progreso</t>
+          <t>Mis cursos y Curso: Últimas dos semanas</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -3328,8 +3336,223 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>US-076</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia de uso</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Usar SIMA cómodamente desde el celular</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>Validada</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Inicio, Mis cursos, Curso y Nueva clase a 390 px de ancho</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Sin desplazamiento horizontal; el menú lateral se reduce a pestañas para que el contenido aparezca primero.</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>US-077</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia de uso</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Crear un curso en una pantalla corta</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>Validada</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Mis cursos → Nuevo curso</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Solo nombre, ciclo, examen, nivel y docente a la vista; temas, objetivo y descripción quedan en «Más detalles».</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>US-078</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia de uso</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Ver las clases del curso y sus acciones sin bajar la página</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E79" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>Validada</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Curso: Nueva clase, Practicar y Repasar arriba; lista de clases primero</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Nivel, opciones de estudio, resumen y progreso pasan a una columna lateral.</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>US-079</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia de uso</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Subir el audio arrastrándolo o grabarlo desde la misma pantalla</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E80" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>Validada</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Nueva clase → Audio</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>Zona para soltar el archivo y grabador con los colores de la marca; el nombre del archivo aparece al elegirlo.</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>US-080</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia de uso</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Leer textos cortos y claros, sin jerga técnica</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>Validada</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Todas las pantallas del estudiante</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>Se retiraron términos como MINI, IRT, θ, backend o prompt de la vista del estudiante; siguen disponibles para el equipo en opciones avanzadas.</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I76"/>
+  <autoFilter ref="A1:I81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3340,7 +3563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3921,30 +4144,58 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Experiencia de uso</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" t="n">
+        <v>19</v>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B21" s="9" t="n">
-        <v>75</v>
-      </c>
-      <c r="C21" s="9" t="n">
-        <v>328</v>
-      </c>
-      <c r="D21" s="9" t="n">
-        <v>61</v>
-      </c>
-      <c r="E21" s="9" t="n">
+      <c r="B22" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>347</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="E22" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="F21" s="9" t="n">
+      <c r="F22" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="G21" s="9" t="n">
+      <c r="G22" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="9" t="n">
+      <c r="H22" s="9" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4121,14 +4372,14 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E6" t="n">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>US-059, US-052, US-050, US-060, US-061, US-062, US-063, US-064, US-065, US-066, US-067, US-068, US-069, US-070, US-071, US-072, US-073, US-074, US-075</t>
+          <t>US-059, US-052, US-050, US-060, US-061, US-062, US-063, US-064, US-065, US-066, US-067, US-068, US-069, US-070, US-071, US-072, US-073, US-074, US-075, US-076, US-077, US-078, US-079, US-080</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mejoras tras la prueba con estudiantes: vocabulario tecnico, resumen completo, conceptos clave y PDF
- Whisper recibe idioma, curso y vocabulario (local, remoto y nube)
- Revision por partes de terminos mal transcritos con validacion y aprendizaje del vocabulario del curso
- Campo Vocabulario en el curso (migracion 0024)
- Resumen de clases largas por partes para cubrir todo el audio; conceptos clave como terminos del area
- Mapa y pagina de la clase toman los conceptos del resumen de la clase
- Descarga de preguntas con hoja de respuestas y de resumenes en PDF (reportlab + DejaVu Sans)
- Plantillas de generacion, coherencia y transcripcion con regla de ortografia
- Servicio de Whisper descarta cuerpos pequenos antes de rechazar el token
</commit_message>
<xml_diff>
--- a/desarollo/PRODUCT BACKLOG_v2_validado.xlsx
+++ b/desarollo/PRODUCT BACKLOG_v2_validado.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backlog validado'!$A$1:$I$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backlog validado'!$A$1:$I$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -988,7 +988,11 @@
           <t>Nueva clase con audio → la clase muestra la transcripción</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Whisper recibe el idioma, el curso y su vocabulario para escribir bien los términos técnicos.</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
@@ -2432,7 +2436,11 @@
           <t>Clase → Mapa</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Tras la prueba con estudiantes, los conceptos clave salen del resumen de la clase y ya no de fragmentos de las preguntas.</t>
+        </is>
+      </c>
       <c r="I53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
@@ -2534,10 +2542,14 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Clase → Resumen</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr"/>
+          <t>Clase → Resumen · Descargar PDF</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Las clases largas se resumen por partes para cubrir todo el audio, no solo el inicio.</t>
+        </is>
+      </c>
       <c r="I56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
@@ -2632,9 +2644,9 @@
       <c r="E59" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>Validada</t>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>Con cambios</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -2644,7 +2656,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Se descarga como «Copia de tus preguntas».</t>
+          <t>Se descarga en PDF con hoja de respuestas, como pidieron los estudiantes; el JSON queda como exportación de datos.</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr"/>
@@ -3551,8 +3563,51 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>US-081</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia de uso</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Ver bien escritos los términos técnicos de mi curso</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>Validada</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Curso → Vocabulario · Clase con audio → Ver estado: términos técnicos revisados</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Un modelo revisa la transcripción por partes y corrige solo términos mal transcritos; los términos técnicos corregidos se suman al vocabulario del curso.</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I81"/>
+  <autoFilter ref="A1:I82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4044,10 +4099,10 @@
         <v>13</v>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -4150,13 +4205,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C21" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -4178,16 +4233,16 @@
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="D22" s="9" t="n">
         <v>66</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F22" s="9" t="n">
         <v>4</v>
@@ -4372,14 +4427,14 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" t="n">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>US-059, US-052, US-050, US-060, US-061, US-062, US-063, US-064, US-065, US-066, US-067, US-068, US-069, US-070, US-071, US-072, US-073, US-074, US-075, US-076, US-077, US-078, US-079, US-080</t>
+          <t>US-059, US-052, US-050, US-060, US-061, US-062, US-063, US-064, US-065, US-066, US-067, US-068, US-069, US-070, US-071, US-072, US-073, US-074, US-075, US-076, US-077, US-078, US-079, US-080, US-081</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Backlog validado: HTTPS en sima.pmoluna.com y transcripcion con Whisper API del equipo
</commit_message>
<xml_diff>
--- a/desarollo/PRODUCT BACKLOG_v2_validado.xlsx
+++ b/desarollo/PRODUCT BACKLOG_v2_validado.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,13 +52,9 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="009B2C2C"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -90,11 +86,6 @@
         <fgColor rgb="00ECECEC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FBE3E3"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -108,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -128,11 +119,8 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1024,12 +1012,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Salud del sistema: transcripción remota alcanzable</t>
+          <t>Diagnóstico: Whisper API lista</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Whisper corre en la PC del equipo y el VPS le envía el audio por un túnel SSH cifrado; ningún tercero recibe el audio.</t>
+          <t>Whisper corre en una PC con GPU del equipo; el VPS le envía el audio por HTTPS (Cloudflare Tunnel) con clave privada.</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
@@ -3327,19 +3315,19 @@
       <c r="E76" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F76" s="7" t="inlineStr">
-        <is>
-          <t>En curso</t>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>Validada</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>http://162.243.33.172:8080</t>
+          <t>https://sima.pmoluna.com</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Publicado en el VPS provisional con la misma pila de la arquitectura objetivo en Azure; falta el subdominio con HTTPS.</t>
+          <t>Publicado con certificado Let's Encrypt en el VPS provisional, con la misma pila de la arquitectura objetivo en Azure; registro por invitación y puerto 8080 cerrado.</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -3625,42 +3613,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Épica</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Validada</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Con cambios</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
-      <c r="G1" s="8" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Reemplazada</t>
         </is>
       </c>
-      <c r="H1" s="8" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>En curso</t>
         </is>
@@ -4183,7 +4171,7 @@
         <v>30</v>
       </c>
       <c r="D20" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -4195,7 +4183,7 @@
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -4227,31 +4215,31 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n">
+      <c r="B22" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="C22" s="9" t="n">
+      <c r="C22" s="8" t="n">
         <v>352</v>
       </c>
-      <c r="D22" s="9" t="n">
-        <v>66</v>
-      </c>
-      <c r="E22" s="9" t="n">
+      <c r="D22" s="8" t="n">
+        <v>67</v>
+      </c>
+      <c r="E22" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="F22" s="9" t="n">
+      <c r="F22" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="G22" s="9" t="n">
+      <c r="G22" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="9" t="n">
-        <v>1</v>
+      <c r="H22" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4277,32 +4265,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Objetivo</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Resultado</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="E1" s="8" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="F1" s="8" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Historias</t>
         </is>

</xml_diff>

<commit_message>
Backlog validado: prueba con estudiantes, seguridad del servidor, dos workers y avance del resumen (85 historias)
</commit_message>
<xml_diff>
--- a/desarollo/PRODUCT BACKLOG_v2_validado.xlsx
+++ b/desarollo/PRODUCT BACKLOG_v2_validado.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leyenda" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backlog validado'!$A$1:$I$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backlog validado'!$A$1:$I$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3120,7 +3120,7 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Worker separado y límite de trabajos pendientes por usuario.</t>
+          <t>La cola vive en la base de datos, con límite de trabajos pendientes por usuario.</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
@@ -3283,10 +3283,14 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Página /salud/ y logs</t>
-        </is>
-      </c>
-      <c r="H75" s="2" t="inlineStr"/>
+          <t>Página /salud/ y diagnóstico check_ai</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>En público solo se ve si la base y la cola responden; los modelos y la transcripción los ve el equipo.</t>
+        </is>
+      </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
@@ -3339,21 +3343,21 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>US-076</t>
+          <t>US-082</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Experiencia de uso</t>
+          <t>Operación y despliegue</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Usar SIMA cómodamente desde el celular</t>
+          <t>Crear cuentas solo con un código de invitación</t>
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>5</v>
@@ -3365,12 +3369,12 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Inicio, Mis cursos, Curso y Nueva clase a 390 px de ancho</t>
+          <t>Crear cuenta → Código de invitación</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Sin desplazamiento horizontal; el menú lateral se reduce a pestañas para que el contenido aparezca primero.</t>
+          <t>Evita que cuentas desconocidas gasten los créditos de IA mientras dura la validación.</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -3382,17 +3386,17 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>US-077</t>
+          <t>US-083</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Experiencia de uso</t>
+          <t>Operación y despliegue</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Crear un curso en una pantalla corta</t>
+          <t>Recibir mi resumen o refuerzo sin esperar a que terminen las clases largas</t>
         </is>
       </c>
       <c r="D78" s="2" t="n">
@@ -3408,12 +3412,12 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Mis cursos → Nuevo curso</t>
+          <t>Generar un resumen mientras otra clase se transcribe</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Solo nombre, ciclo, examen, nivel y docente a la vista; temas, objetivo y descripción quedan en «Más detalles».</t>
+          <t>Dos workers: uno para clases y otro para resúmenes y refuerzos, cada uno con tope de memoria.</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -3425,17 +3429,17 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>US-078</t>
+          <t>US-085</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Experiencia de uso</t>
+          <t>Operación y despliegue</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Ver las clases del curso y sus acciones sin bajar la página</t>
+          <t>Transcribir los audios en la GPU del equipo sin cargar el servidor</t>
         </is>
       </c>
       <c r="D79" s="2" t="n">
@@ -3451,12 +3455,12 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Curso: Nueva clase, Practicar y Repasar arriba; lista de clases primero</t>
+          <t>Clase con audio → Ver estado: Audio enviado a Whisper API</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>Nivel, opciones de estudio, resumen y progreso pasan a una columna lateral.</t>
+          <t>El servidor envía el audio por HTTPS a la Whisper API del equipo con una clave privada; si el servicio se corta, retoma el mismo trabajo.</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
@@ -3468,7 +3472,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>US-079</t>
+          <t>US-076</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -3478,11 +3482,11 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Subir el audio arrastrándolo o grabarlo desde la misma pantalla</t>
+          <t>Usar SIMA cómodamente desde el celular</t>
         </is>
       </c>
       <c r="D80" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>5</v>
@@ -3494,12 +3498,12 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Nueva clase → Audio</t>
+          <t>Inicio, Mis cursos, Curso y Nueva clase a 390 px de ancho</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Zona para soltar el archivo y grabador con los colores de la marca; el nombre del archivo aparece al elegirlo.</t>
+          <t>Sin desplazamiento horizontal; el menú lateral se reduce a pestañas para que el contenido aparezca primero.</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
@@ -3511,7 +3515,7 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>US-080</t>
+          <t>US-077</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -3521,7 +3525,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Leer textos cortos y claros, sin jerga técnica</t>
+          <t>Crear un curso en una pantalla corta</t>
         </is>
       </c>
       <c r="D81" s="2" t="n">
@@ -3537,12 +3541,12 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Todas las pantallas del estudiante</t>
+          <t>Mis cursos → Nuevo curso</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Se retiraron términos como MINI, IRT, θ, backend o prompt de la vista del estudiante; siguen disponibles para el equipo en opciones avanzadas.</t>
+          <t>Solo nombre, ciclo, examen, nivel y docente a la vista; temas, objetivo y descripción quedan en «Más detalles».</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr">
@@ -3554,48 +3558,220 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
+          <t>US-078</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia de uso</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Ver las clases del curso y sus acciones sin bajar la página</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>Validada</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Curso: Nueva clase, Practicar y Repasar arriba; lista de clases primero</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Nivel, opciones de estudio, resumen y progreso pasan a una columna lateral.</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>US-079</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia de uso</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Subir el audio arrastrándolo o grabarlo desde la misma pantalla</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>Validada</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Nueva clase → Audio</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>Zona para soltar el archivo y grabador con los colores de la marca; el nombre del archivo aparece al elegirlo.</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>US-080</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia de uso</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Leer textos cortos y claros, sin jerga técnica</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>Validada</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Todas las pantallas del estudiante</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Se retiraron términos como MINI, IRT, θ, backend o prompt de la vista del estudiante; siguen disponibles para el equipo en opciones avanzadas.</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
           <t>US-081</t>
         </is>
       </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="B85" s="2" t="inlineStr">
         <is>
           <t>Experiencia de uso</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
+      <c r="C85" s="2" t="inlineStr">
         <is>
           <t>Ver bien escritos los términos técnicos de mi curso</t>
         </is>
       </c>
-      <c r="D82" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E82" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="F82" s="3" t="inlineStr">
-        <is>
-          <t>Validada</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr">
+      <c r="D85" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E85" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>Validada</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
         <is>
           <t>Curso → Vocabulario · Clase con audio → Ver estado: términos técnicos revisados</t>
         </is>
       </c>
-      <c r="H82" s="2" t="inlineStr">
+      <c r="H85" s="2" t="inlineStr">
         <is>
           <t>Un modelo revisa la transcripción por partes y corrige solo términos mal transcritos; los términos técnicos corregidos se suman al vocabulario del curso.</t>
         </is>
       </c>
-      <c r="I82" s="2" t="inlineStr">
+      <c r="I85" s="2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>US-084</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Experiencia de uso</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Ver en qué va mi resumen mientras se genera</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>Validada</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Clase → Resumen → Generar: tarjeta de avance</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Muestra si está en cola o qué parte de la clase está leyendo; la página se actualiza sola.</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I82"/>
+  <autoFilter ref="A1:I86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4165,13 +4341,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C20" t="n">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="D20" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -4193,13 +4369,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C21" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -4221,13 +4397,13 @@
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C22" s="8" t="n">
-        <v>352</v>
+        <v>365</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E22" s="8" t="n">
         <v>9</v>
@@ -4406,23 +4582,23 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Motor adaptativo v2 y operación</t>
+          <t>Motor adaptativo v2, operación y prueba con estudiantes</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Práctica por curso, refuerzo, repaso, resúmenes, cola persistente y despliegue.</t>
+          <t>Práctica por curso, refuerzo, repaso, resúmenes, despliegue con HTTPS y mejoras tras probarla con estudiantes.</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E6" t="n">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>US-059, US-052, US-050, US-060, US-061, US-062, US-063, US-064, US-065, US-066, US-067, US-068, US-069, US-070, US-071, US-072, US-073, US-074, US-075, US-076, US-077, US-078, US-079, US-080, US-081</t>
+          <t>US-059, US-052, US-050, US-060, US-061, US-062, US-063, US-064, US-065, US-066, US-067, US-068, US-069, US-070, US-071, US-072, US-073, US-074, US-075, US-076, US-077, US-078, US-079, US-080, US-084, US-081, US-082, US-083, US-085</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Backlog validado: redaccion formal de observaciones
</commit_message>
<xml_diff>
--- a/desarollo/PRODUCT BACKLOG_v2_validado.xlsx
+++ b/desarollo/PRODUCT BACKLOG_v2_validado.xlsx
@@ -2426,7 +2426,7 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Tras la prueba con estudiantes, los conceptos clave salen del resumen de la clase y ya no de fragmentos de las preguntas.</t>
+          <t>A partir de la prueba con estudiantes, los conceptos clave se obtienen del resumen de la clase y no de fragmentos de las preguntas.</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr"/>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Se descarga en PDF con hoja de respuestas, como pidieron los estudiantes; el JSON queda como exportación de datos.</t>
+          <t>Se descarga en PDF con hoja de respuestas; el JSON se mantiene como exportación de datos.</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr"/>
@@ -3288,7 +3288,7 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>En público solo se ve si la base y la cola responden; los modelos y la transcripción los ve el equipo.</t>
+          <t>La vista pública solo informa el estado de la base de datos y la cola; el detalle técnico queda reservado al equipo.</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Evita que cuentas desconocidas gasten los créditos de IA mientras dura la validación.</t>
+          <t>Restringe el consumo de créditos de IA a usuarios autorizados durante la validación.</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Práctica por curso, refuerzo, repaso, resúmenes, despliegue con HTTPS y mejoras tras probarla con estudiantes.</t>
+          <t>Práctica por curso, refuerzo, repaso, resúmenes, despliegue con HTTPS y mejoras derivadas de la prueba con estudiantes.</t>
         </is>
       </c>
       <c r="D6" t="n">

</xml_diff>